<commit_message>
docs: update stack spec for Kubernetes target and UI/UX design
Revises the deployment target from docker-compose-on-a-VPS to
per-repo Docker images deployed via Kubernetes manifests, and adds
the responsive web/mobile UI/UX design section. Also picks up the
latest save of the source spreadsheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Idea/Catatan_HPP_Keuangan_Bisnis.xlsx
+++ b/Idea/Catatan_HPP_Keuangan_Bisnis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\App\Idea\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\App\stock-business-analyst\Idea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D191ABA-3C8D-48E4-A8B8-41141B0640AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB0F333-3474-4ACE-ADDB-4512808E2489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Penjualan" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="91">
   <si>
     <t>CATATAN PENJUALAN</t>
   </si>
@@ -204,120 +204,6 @@
   </si>
   <si>
     <t>Nilai Persediaan</t>
-  </si>
-  <si>
-    <t>[Black] Croco Nocturne Bag</t>
-  </si>
-  <si>
-    <t>pcs</t>
-  </si>
-  <si>
-    <t>[Dark Brown] Croco Nocturne Bag</t>
-  </si>
-  <si>
-    <t>[Maroon] Croco Nocturne Bag</t>
-  </si>
-  <si>
-    <t>[Blue Denim] Croco Nocturne Bag</t>
-  </si>
-  <si>
-    <t>[Black] Croco Sonnet Bag</t>
-  </si>
-  <si>
-    <t>[Dark Brown] Croco Sonnet Bag</t>
-  </si>
-  <si>
-    <t>[Maroon] Croco Sonnet Bag</t>
-  </si>
-  <si>
-    <t>[Blue Denim] Croco Sonnet Bag</t>
-  </si>
-  <si>
-    <t>Accessories Anggur</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Baby - Biru</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Baby - Hitam</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Baby - Putih</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Baby - Pink</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Baby - Mocca</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Baby - Maroon</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Girl - Pink</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Girl - Hitam</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Girl - Biru</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Girl - Mocca</t>
-  </si>
-  <si>
-    <t>Acc - Sleeping Girl - Putih</t>
-  </si>
-  <si>
-    <t>Thank You Card</t>
-  </si>
-  <si>
-    <t>Silica Gel - 5gr</t>
-  </si>
-  <si>
-    <t>Air Bag - 20x30</t>
-  </si>
-  <si>
-    <t>Bubble Wrap - 10x60</t>
-  </si>
-  <si>
-    <t>roll</t>
-  </si>
-  <si>
-    <t>Bubble Wrap - 125x50</t>
-  </si>
-  <si>
-    <t>Plastic Wrap - 50x300</t>
-  </si>
-  <si>
-    <t>Dust Bag Putih Custom - 40x30</t>
-  </si>
-  <si>
-    <t>Dust Bag Putih Custom - 50x50</t>
-  </si>
-  <si>
-    <t>Polymailer - 30x40</t>
-  </si>
-  <si>
-    <t>Polymailer - 40x60</t>
-  </si>
-  <si>
-    <t>Box Kardus - 27x20x14,5cm</t>
-  </si>
-  <si>
-    <t>Box Kardus - 32x22x11,5cm</t>
-  </si>
-  <si>
-    <t>Box Pizza - 30x20x5cm</t>
-  </si>
-  <si>
-    <t>Sticker Custom</t>
-  </si>
-  <si>
-    <t>Cup Saos - 35ml</t>
-  </si>
-  <si>
-    <t>Kertas Tisu (30x55cm)</t>
   </si>
   <si>
     <t>TOTAL NILAI PERSEDIAAN</t>
@@ -2545,9 +2431,7 @@
       <c r="E6" s="13">
         <v>0</v>
       </c>
-      <c r="F6" s="14">
-        <v>9310000</v>
-      </c>
+      <c r="F6" s="14"/>
       <c r="G6" s="13">
         <v>0</v>
       </c>
@@ -2574,7 +2458,7 @@
       </c>
       <c r="O6" s="5">
         <f t="shared" si="0"/>
-        <v>9310000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -2788,7 +2672,7 @@
       </c>
       <c r="F11" s="16">
         <f t="shared" si="1"/>
-        <v>9310000</v>
+        <v>0</v>
       </c>
       <c r="G11" s="8">
         <f t="shared" si="1"/>
@@ -2824,7 +2708,7 @@
       </c>
       <c r="O11" s="8">
         <f t="shared" si="1"/>
-        <v>9310000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2897,7 +2781,7 @@
       </c>
       <c r="F14" s="21">
         <f t="shared" si="2"/>
-        <v>9310000</v>
+        <v>0</v>
       </c>
       <c r="G14" s="20">
         <f t="shared" si="2"/>
@@ -2933,7 +2817,7 @@
       </c>
       <c r="O14" s="20">
         <f t="shared" si="2"/>
-        <v>9310000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -8270,12 +8154,8 @@
       <c r="E10" s="4">
         <v>0</v>
       </c>
-      <c r="F10" s="4">
-        <v>13177790</v>
-      </c>
-      <c r="G10" s="4">
-        <v>946000</v>
-      </c>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
       <c r="H10" s="4">
         <v>0</v>
       </c>
@@ -8299,7 +8179,7 @@
       </c>
       <c r="O10" s="5">
         <f t="shared" si="0"/>
-        <v>14123790</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -8513,11 +8393,11 @@
       </c>
       <c r="F15" s="8">
         <f t="shared" si="1"/>
-        <v>13177790</v>
+        <v>0</v>
       </c>
       <c r="G15" s="8">
         <f t="shared" si="1"/>
-        <v>946000</v>
+        <v>0</v>
       </c>
       <c r="H15" s="8">
         <f t="shared" si="1"/>
@@ -8549,7 +8429,7 @@
       </c>
       <c r="O15" s="8">
         <f t="shared" si="1"/>
-        <v>14123790</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
@@ -9687,17 +9567,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
       <c r="D5" s="31">
-        <v>58000</v>
+        <v>0</v>
       </c>
       <c r="E5" s="32">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F5" s="32">
         <v>0</v>
@@ -9707,26 +9583,22 @@
       </c>
       <c r="H5" s="33">
         <f t="shared" ref="H5:H68" si="0">E5+F5-G5</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I5" s="34">
         <f t="shared" ref="I5:I68" si="1">H5*D5</f>
-        <v>1160000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
       <c r="D6" s="31">
-        <v>58000</v>
+        <v>0</v>
       </c>
       <c r="E6" s="32">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F6" s="32">
         <v>0</v>
@@ -9736,26 +9608,22 @@
       </c>
       <c r="H6" s="33">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="I6" s="34">
         <f t="shared" si="1"/>
-        <v>1044000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
       <c r="D7" s="31">
-        <v>58000</v>
+        <v>0</v>
       </c>
       <c r="E7" s="32">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F7" s="32">
         <v>0</v>
@@ -9765,26 +9633,22 @@
       </c>
       <c r="H7" s="33">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I7" s="34">
         <f t="shared" si="1"/>
-        <v>1102000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
       <c r="D8" s="31">
-        <v>58000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="32">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F8" s="32">
         <v>0</v>
@@ -9794,11 +9658,11 @@
       </c>
       <c r="H8" s="33">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I8" s="34">
         <f t="shared" si="1"/>
-        <v>1160000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -9828,14 +9692,10 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
       <c r="D10" s="31">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="32">
         <v>0</v>
@@ -9857,14 +9717,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
       <c r="D11" s="31">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="32">
         <v>0</v>
@@ -9886,14 +9742,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
       <c r="D12" s="31">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="E12" s="32">
         <v>0</v>
@@ -9915,14 +9767,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
       <c r="D13" s="31">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="E13" s="32">
         <v>0</v>
@@ -10169,17 +10017,13 @@
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
       <c r="D23" s="31">
-        <v>7500</v>
+        <v>0</v>
       </c>
       <c r="E23" s="32">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F23" s="32">
         <v>0</v>
@@ -10189,25 +10033,21 @@
       </c>
       <c r="H23" s="33">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="I23" s="34">
         <f t="shared" si="1"/>
-        <v>180000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="C24" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
       <c r="D24" s="31">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="E24" s="32">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F24" s="32">
         <v>0</v>
@@ -10217,25 +10057,21 @@
       </c>
       <c r="H24" s="33">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I24" s="34">
         <f t="shared" si="1"/>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
       <c r="D25" s="31">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="E25" s="32">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F25" s="32">
         <v>0</v>
@@ -10245,25 +10081,21 @@
       </c>
       <c r="H25" s="33">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I25" s="34">
         <f t="shared" si="1"/>
-        <v>54000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B26" s="30"/>
+      <c r="C26" s="30"/>
       <c r="D26" s="31">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="E26" s="32">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F26" s="32">
         <v>0</v>
@@ -10273,25 +10105,21 @@
       </c>
       <c r="H26" s="33">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I26" s="34">
         <f t="shared" si="1"/>
-        <v>54000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="30" t="s">
-        <v>71</v>
-      </c>
-      <c r="C27" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
       <c r="D27" s="31">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="E27" s="32">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F27" s="32">
         <v>0</v>
@@ -10301,25 +10129,21 @@
       </c>
       <c r="H27" s="33">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I27" s="34">
         <f t="shared" si="1"/>
-        <v>99000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="C28" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B28" s="30"/>
+      <c r="C28" s="30"/>
       <c r="D28" s="31">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="E28" s="32">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F28" s="32">
         <v>0</v>
@@ -10329,25 +10153,21 @@
       </c>
       <c r="H28" s="33">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I28" s="34">
         <f t="shared" si="1"/>
-        <v>72000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B29" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="C29" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
       <c r="D29" s="31">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="E29" s="32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F29" s="32">
         <v>0</v>
@@ -10357,25 +10177,21 @@
       </c>
       <c r="H29" s="33">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I29" s="34">
         <f t="shared" si="1"/>
-        <v>81000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
       <c r="D30" s="31">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="E30" s="32">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F30" s="32">
         <v>0</v>
@@ -10385,25 +10201,21 @@
       </c>
       <c r="H30" s="33">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I30" s="34">
         <f t="shared" si="1"/>
-        <v>132000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B31" s="30"/>
+      <c r="C31" s="30"/>
       <c r="D31" s="31">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="E31" s="32">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F31" s="32">
         <v>0</v>
@@ -10413,25 +10225,21 @@
       </c>
       <c r="H31" s="33">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I31" s="34">
         <f t="shared" si="1"/>
-        <v>144000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="C32" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B32" s="30"/>
+      <c r="C32" s="30"/>
       <c r="D32" s="31">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="E32" s="32">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F32" s="32">
         <v>0</v>
@@ -10441,25 +10249,21 @@
       </c>
       <c r="H32" s="33">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I32" s="34">
         <f t="shared" si="1"/>
-        <v>132000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B33" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="C33" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B33" s="30"/>
+      <c r="C33" s="30"/>
       <c r="D33" s="31">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="E33" s="32">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F33" s="32">
         <v>0</v>
@@ -10469,25 +10273,21 @@
       </c>
       <c r="H33" s="33">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I33" s="34">
         <f t="shared" si="1"/>
-        <v>132000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
       <c r="D34" s="31">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="E34" s="32">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F34" s="32">
         <v>0</v>
@@ -10497,17 +10297,19 @@
       </c>
       <c r="H34" s="33">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I34" s="34">
         <f t="shared" si="1"/>
-        <v>144000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B35" s="30"/>
       <c r="C35" s="30"/>
-      <c r="D35" s="31"/>
+      <c r="D35" s="31">
+        <v>0</v>
+      </c>
       <c r="E35" s="32">
         <v>0</v>
       </c>
@@ -10529,7 +10331,9 @@
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B36" s="30"/>
       <c r="C36" s="30"/>
-      <c r="D36" s="31"/>
+      <c r="D36" s="31">
+        <v>0</v>
+      </c>
       <c r="E36" s="32">
         <v>0</v>
       </c>
@@ -10549,17 +10353,13 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="30" t="s">
-        <v>79</v>
-      </c>
-      <c r="C37" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B37" s="30"/>
+      <c r="C37" s="30"/>
       <c r="D37" s="31">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E37" s="32">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="F37" s="32">
         <v>0</v>
@@ -10569,26 +10369,22 @@
       </c>
       <c r="H37" s="33">
         <f t="shared" si="0"/>
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="I37" s="34">
         <f t="shared" si="1"/>
-        <v>230000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="C38" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
       <c r="D38" s="31">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="E38" s="32">
-        <v>360</v>
+        <v>0</v>
       </c>
       <c r="F38" s="32">
         <v>0</v>
@@ -10598,26 +10394,22 @@
       </c>
       <c r="H38" s="33">
         <f t="shared" si="0"/>
-        <v>360</v>
+        <v>0</v>
       </c>
       <c r="I38" s="34">
         <f t="shared" si="1"/>
-        <v>61920</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
-      <c r="B39" s="30" t="s">
-        <v>81</v>
-      </c>
-      <c r="C39" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
       <c r="D39" s="31">
-        <v>834</v>
+        <v>0</v>
       </c>
       <c r="E39" s="32">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F39" s="32">
         <v>0</v>
@@ -10627,26 +10419,22 @@
       </c>
       <c r="H39" s="33">
         <f t="shared" si="0"/>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I39" s="34">
         <f t="shared" si="1"/>
-        <v>166800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="C40" s="30" t="s">
-        <v>83</v>
-      </c>
+      <c r="B40" s="30"/>
+      <c r="C40" s="30"/>
       <c r="D40" s="31">
-        <v>29500</v>
+        <v>0</v>
       </c>
       <c r="E40" s="32">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F40" s="32">
         <v>0</v>
@@ -10656,26 +10444,22 @@
       </c>
       <c r="H40" s="33">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I40" s="34">
         <f t="shared" si="1"/>
-        <v>118000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
-      <c r="B41" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="C41" s="30" t="s">
-        <v>83</v>
-      </c>
+      <c r="B41" s="30"/>
+      <c r="C41" s="30"/>
       <c r="D41" s="31">
-        <v>180000</v>
+        <v>0</v>
       </c>
       <c r="E41" s="32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F41" s="32">
         <v>0</v>
@@ -10685,24 +10469,22 @@
       </c>
       <c r="H41" s="33">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I41" s="34">
         <f t="shared" si="1"/>
-        <v>360000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
-      <c r="B42" s="30" t="s">
-        <v>85</v>
-      </c>
+      <c r="B42" s="30"/>
       <c r="C42" s="30"/>
       <c r="D42" s="31">
-        <v>146800</v>
+        <v>0</v>
       </c>
       <c r="E42" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" s="32">
         <v>0</v>
@@ -10712,26 +10494,22 @@
       </c>
       <c r="H42" s="33">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42" s="34">
         <f t="shared" si="1"/>
-        <v>146800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
-      <c r="B43" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="C43" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B43" s="30"/>
+      <c r="C43" s="30"/>
       <c r="D43" s="31">
-        <v>4150</v>
+        <v>0</v>
       </c>
       <c r="E43" s="32">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F43" s="32">
         <v>0</v>
@@ -10741,26 +10519,22 @@
       </c>
       <c r="H43" s="33">
         <f t="shared" si="0"/>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I43" s="34">
         <f t="shared" si="1"/>
-        <v>830000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
-      <c r="B44" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="C44" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B44" s="30"/>
+      <c r="C44" s="30"/>
       <c r="D44" s="31">
-        <v>5930</v>
+        <v>0</v>
       </c>
       <c r="E44" s="32">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F44" s="32">
         <v>0</v>
@@ -10770,26 +10544,22 @@
       </c>
       <c r="H44" s="33">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I44" s="34">
         <f t="shared" si="1"/>
-        <v>593000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
-      <c r="B45" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="C45" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B45" s="30"/>
+      <c r="C45" s="30"/>
       <c r="D45" s="31">
-        <v>307</v>
+        <v>0</v>
       </c>
       <c r="E45" s="32">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="F45" s="32">
         <v>0</v>
@@ -10799,26 +10569,22 @@
       </c>
       <c r="H45" s="33">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I45" s="34">
         <f t="shared" si="1"/>
-        <v>92100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
-      <c r="B46" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="C46" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B46" s="30"/>
+      <c r="C46" s="30"/>
       <c r="D46" s="31">
-        <v>958</v>
+        <v>0</v>
       </c>
       <c r="E46" s="32">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F46" s="32">
         <v>0</v>
@@ -10828,26 +10594,22 @@
       </c>
       <c r="H46" s="33">
         <f t="shared" si="0"/>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I46" s="34">
         <f t="shared" si="1"/>
-        <v>191600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
-      <c r="B47" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C47" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B47" s="30"/>
+      <c r="C47" s="30"/>
       <c r="D47" s="31">
-        <v>2530</v>
+        <v>0</v>
       </c>
       <c r="E47" s="32">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F47" s="32">
         <v>0</v>
@@ -10857,26 +10619,22 @@
       </c>
       <c r="H47" s="33">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I47" s="34">
         <f t="shared" si="1"/>
-        <v>126500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
-      <c r="B48" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="C48" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B48" s="30"/>
+      <c r="C48" s="30"/>
       <c r="D48" s="31">
-        <v>2890</v>
+        <v>0</v>
       </c>
       <c r="E48" s="32">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F48" s="32">
         <v>0</v>
@@ -10886,26 +10644,22 @@
       </c>
       <c r="H48" s="33">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I48" s="34">
         <f t="shared" si="1"/>
-        <v>144500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
-      <c r="B49" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="C49" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B49" s="30"/>
+      <c r="C49" s="30"/>
       <c r="D49" s="31">
-        <v>1955</v>
+        <v>0</v>
       </c>
       <c r="E49" s="32">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F49" s="32">
         <v>0</v>
@@ -10915,26 +10669,22 @@
       </c>
       <c r="H49" s="33">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I49" s="34">
         <f t="shared" si="1"/>
-        <v>195500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
-      <c r="B50" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="C50" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B50" s="30"/>
+      <c r="C50" s="30"/>
       <c r="D50" s="31">
-        <v>933</v>
+        <v>0</v>
       </c>
       <c r="E50" s="32">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F50" s="32">
         <v>0</v>
@@ -10944,55 +10694,47 @@
       </c>
       <c r="H50" s="33">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="I50" s="34">
         <f t="shared" si="1"/>
-        <v>139950</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
-      <c r="B51" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="C51" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B51" s="30"/>
+      <c r="C51" s="30"/>
       <c r="D51" s="31">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="E51" s="32">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F51" s="32">
         <v>0</v>
       </c>
       <c r="G51" s="32">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H51" s="33">
         <f t="shared" si="0"/>
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="I51" s="34">
         <f t="shared" si="1"/>
-        <v>24700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
-      <c r="B52" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="C52" s="30" t="s">
-        <v>59</v>
-      </c>
+      <c r="B52" s="30"/>
+      <c r="C52" s="30"/>
       <c r="D52" s="31">
-        <v>244</v>
+        <v>0</v>
       </c>
       <c r="E52" s="32">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="F52" s="32">
         <v>0</v>
@@ -11002,11 +10744,11 @@
       </c>
       <c r="H52" s="33">
         <f t="shared" si="0"/>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I52" s="34">
         <f t="shared" si="1"/>
-        <v>61000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11432,7 +11174,7 @@
     <row r="71" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6"/>
       <c r="B71" s="35" t="s">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="C71" s="36"/>
       <c r="D71" s="37"/>
@@ -11442,7 +11184,7 @@
       <c r="H71" s="38"/>
       <c r="I71" s="39">
         <f>SUM(I5:I70)</f>
-        <v>9262370</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -20772,7 +20514,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="18" x14ac:dyDescent="0.25">
       <c r="B1" s="60" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="C1" s="54"/>
       <c r="D1" s="54"/>
@@ -20807,7 +20549,7 @@
     <row r="4" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="40"/>
       <c r="B4" s="40" t="s">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="C4" s="40" t="s">
         <v>4</v>
@@ -20852,7 +20594,7 @@
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
       <c r="B5" s="41" t="s">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="C5" s="42">
         <f>Penjualan!C10</f>
@@ -20910,7 +20652,7 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="15"/>
       <c r="B6" s="41" t="s">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="C6" s="42">
         <f>HPP!C14</f>
@@ -20926,7 +20668,7 @@
       </c>
       <c r="F6" s="42">
         <f>HPP!F14</f>
-        <v>9310000</v>
+        <v>0</v>
       </c>
       <c r="G6" s="42">
         <f>HPP!G14</f>
@@ -20962,13 +20704,13 @@
       </c>
       <c r="O6" s="42">
         <f>HPP!O14</f>
-        <v>9310000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="43"/>
       <c r="B8" s="44" t="s">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="C8" s="45">
         <f t="shared" ref="C8:O8" si="0">C5-C6</f>
@@ -20984,7 +20726,7 @@
       </c>
       <c r="F8" s="45">
         <f t="shared" si="0"/>
-        <v>-9310000</v>
+        <v>0</v>
       </c>
       <c r="G8" s="45">
         <f t="shared" si="0"/>
@@ -21020,13 +20762,13 @@
       </c>
       <c r="O8" s="45">
         <f t="shared" si="0"/>
-        <v>-9310000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="46" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="C9" s="47">
         <f t="shared" ref="C9:O9" si="1">IF(C5=0,0,C8/C5)</f>
@@ -21084,7 +20826,7 @@
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="41" t="s">
-        <v>103</v>
+        <v>65</v>
       </c>
       <c r="C11" s="42">
         <f>'Biaya Operasional'!C15</f>
@@ -21100,11 +20842,11 @@
       </c>
       <c r="F11" s="42">
         <f>'Biaya Operasional'!F15</f>
-        <v>13177790</v>
+        <v>0</v>
       </c>
       <c r="G11" s="42">
         <f>'Biaya Operasional'!G15</f>
-        <v>946000</v>
+        <v>0</v>
       </c>
       <c r="H11" s="42">
         <f>'Biaya Operasional'!H15</f>
@@ -21136,13 +20878,13 @@
       </c>
       <c r="O11" s="42">
         <f>'Biaya Operasional'!O15</f>
-        <v>14123790</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="48" t="s">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="C13" s="49">
         <f t="shared" ref="C13:O13" si="2">C8-C11</f>
@@ -21158,11 +20900,11 @@
       </c>
       <c r="F13" s="49">
         <f t="shared" si="2"/>
-        <v>-22487790</v>
+        <v>0</v>
       </c>
       <c r="G13" s="49">
         <f t="shared" si="2"/>
-        <v>-946000</v>
+        <v>0</v>
       </c>
       <c r="H13" s="49">
         <f t="shared" si="2"/>
@@ -21194,13 +20936,13 @@
       </c>
       <c r="O13" s="49">
         <f t="shared" si="2"/>
-        <v>-23433790</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="46" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="C14" s="47">
         <f t="shared" ref="C14:O14" si="3">IF(C5=0,0,C13/C5)</f>
@@ -22260,119 +22002,119 @@
   <sheetData>
     <row r="1" spans="2:2" ht="18" x14ac:dyDescent="0.25">
       <c r="B1" s="50" t="s">
-        <v>106</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="51" t="s">
-        <v>107</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="52" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="52" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="51" t="s">
-        <v>110</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="52" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="52" t="s">
-        <v>112</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="51" t="s">
-        <v>113</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="52" t="s">
-        <v>114</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="52" t="s">
-        <v>115</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="51" t="s">
-        <v>116</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="52" t="s">
-        <v>117</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="51" t="s">
-        <v>118</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="52" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="52" t="s">
-        <v>120</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="52" t="s">
-        <v>121</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="51" t="s">
-        <v>122</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="52" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="52" t="s">
-        <v>124</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="51" t="s">
-        <v>125</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="52" t="s">
-        <v>126</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="52" t="s">
-        <v>127</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="52" t="s">
-        <v>128</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>